<commit_message>
Give the simulation tool bar a much need glow-up
</commit_message>
<xml_diff>
--- a/bitstream/XC2064_output.xlsx
+++ b/bitstream/XC2064_output.xlsx
@@ -1173,12 +1173,12 @@
           <t>IOB P40.O MuxBit: 3</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AT1" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G6</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AU1" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G7</t>
         </is>
@@ -1453,12 +1453,12 @@
           <t>IOB P33.O MuxBit: 3</t>
         </is>
       </c>
-      <c r="CX1" t="inlineStr">
+      <c r="CX1" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G6</t>
         </is>
       </c>
-      <c r="CY1" t="inlineStr">
+      <c r="CY1" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G7</t>
         </is>
@@ -1980,7 +1980,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AU2" t="inlineStr">
+      <c r="AU2" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G9</t>
         </is>
@@ -2260,7 +2260,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CY2" t="inlineStr">
+      <c r="CY2" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G9</t>
         </is>
@@ -4381,12 +4381,12 @@
           <t>CLB HG Logic Table: 1 Bit: 1</t>
         </is>
       </c>
-      <c r="AT5" t="inlineStr">
+      <c r="AT5" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G28</t>
         </is>
       </c>
-      <c r="AU5" t="inlineStr">
+      <c r="AU5" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G10</t>
         </is>
@@ -4661,12 +4661,12 @@
           <t>CLB HD Logic Table: 1 Bit: 1</t>
         </is>
       </c>
-      <c r="CX5" t="inlineStr">
+      <c r="CX5" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G28</t>
         </is>
       </c>
-      <c r="CY5" t="inlineStr">
+      <c r="CY5" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G10</t>
         </is>
@@ -6677,12 +6677,12 @@
           <t>CLB HH</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr">
+      <c r="X8" s="2" t="inlineStr">
         <is>
           <t>CLB HH.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="Y8" t="inlineStr">
+      <c r="Y8" s="2" t="inlineStr">
         <is>
           <t>CLB HH.K MuxBit: 1</t>
         </is>
@@ -6767,12 +6767,12 @@
           <t>CLB HG</t>
         </is>
       </c>
-      <c r="AP8" t="inlineStr">
+      <c r="AP8" s="2" t="inlineStr">
         <is>
           <t>CLB HG.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="AQ8" t="inlineStr">
+      <c r="AQ8" s="2" t="inlineStr">
         <is>
           <t>CLB HG.K MuxBit: 1</t>
         </is>
@@ -6787,12 +6787,12 @@
           <t>PIP  127G18</t>
         </is>
       </c>
-      <c r="AT8" t="inlineStr">
+      <c r="AT8" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G27</t>
         </is>
       </c>
-      <c r="AU8" t="inlineStr">
+      <c r="AU8" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G31</t>
         </is>
@@ -6867,12 +6867,12 @@
           <t>CLB HF</t>
         </is>
       </c>
-      <c r="BJ8" t="inlineStr">
+      <c r="BJ8" s="2" t="inlineStr">
         <is>
           <t>CLB HF.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="BK8" t="inlineStr">
+      <c r="BK8" s="2" t="inlineStr">
         <is>
           <t>CLB HF.K MuxBit: 1</t>
         </is>
@@ -6957,12 +6957,12 @@
           <t>CLB HE</t>
         </is>
       </c>
-      <c r="CB8" t="inlineStr">
+      <c r="CB8" s="2" t="inlineStr">
         <is>
           <t>CLB HE.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="CC8" t="inlineStr">
+      <c r="CC8" s="2" t="inlineStr">
         <is>
           <t>CLB HE.K MuxBit: 1</t>
         </is>
@@ -7047,12 +7047,12 @@
           <t>CLB HD</t>
         </is>
       </c>
-      <c r="CT8" t="inlineStr">
+      <c r="CT8" s="2" t="inlineStr">
         <is>
           <t>CLB HD.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="CU8" t="inlineStr">
+      <c r="CU8" s="2" t="inlineStr">
         <is>
           <t>CLB HD.K MuxBit: 1</t>
         </is>
@@ -7067,12 +7067,12 @@
           <t>PIP  67G18</t>
         </is>
       </c>
-      <c r="CX8" t="inlineStr">
+      <c r="CX8" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G27</t>
         </is>
       </c>
-      <c r="CY8" t="inlineStr">
+      <c r="CY8" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G31</t>
         </is>
@@ -7147,12 +7147,12 @@
           <t>CLB HC</t>
         </is>
       </c>
-      <c r="DN8" t="inlineStr">
+      <c r="DN8" s="2" t="inlineStr">
         <is>
           <t>CLB HC.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="DO8" t="inlineStr">
+      <c r="DO8" s="2" t="inlineStr">
         <is>
           <t>CLB HC.K MuxBit: 1</t>
         </is>
@@ -7237,12 +7237,12 @@
           <t>CLB HB</t>
         </is>
       </c>
-      <c r="EF8" t="inlineStr">
+      <c r="EF8" s="2" t="inlineStr">
         <is>
           <t>CLB HB.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="EG8" t="inlineStr">
+      <c r="EG8" s="2" t="inlineStr">
         <is>
           <t>CLB HB.K MuxBit: 1</t>
         </is>
@@ -7327,12 +7327,12 @@
           <t>CLB HA</t>
         </is>
       </c>
-      <c r="EX8" t="inlineStr">
+      <c r="EX8" s="2" t="inlineStr">
         <is>
           <t>CLB HA.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="EY8" t="inlineStr">
+      <c r="EY8" s="2" t="inlineStr">
         <is>
           <t>CLB HA.K MuxBit: 1</t>
         </is>
@@ -10000,7 +10000,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AU12" t="inlineStr">
+      <c r="AU12" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G30</t>
         </is>
@@ -10280,7 +10280,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CY12" t="inlineStr">
+      <c r="CY12" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G30</t>
         </is>
@@ -10797,7 +10797,7 @@
           <t>CLB GG Logic Table: 1 Bit: 1</t>
         </is>
       </c>
-      <c r="AT13" t="inlineStr">
+      <c r="AT13" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G47</t>
         </is>
@@ -11077,7 +11077,7 @@
           <t>CLB GD Logic Table: 1 Bit: 1</t>
         </is>
       </c>
-      <c r="CX13" t="inlineStr">
+      <c r="CX13" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G47</t>
         </is>
@@ -13093,12 +13093,12 @@
           <t>CLB GH</t>
         </is>
       </c>
-      <c r="X16" t="inlineStr">
+      <c r="X16" s="2" t="inlineStr">
         <is>
           <t>CLB GH.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="Y16" t="inlineStr">
+      <c r="Y16" s="2" t="inlineStr">
         <is>
           <t>CLB GH.K MuxBit: 1</t>
         </is>
@@ -13183,12 +13183,12 @@
           <t>CLB GG</t>
         </is>
       </c>
-      <c r="AP16" t="inlineStr">
+      <c r="AP16" s="2" t="inlineStr">
         <is>
           <t>CLB GG.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="AQ16" t="inlineStr">
+      <c r="AQ16" s="2" t="inlineStr">
         <is>
           <t>CLB GG.K MuxBit: 1</t>
         </is>
@@ -13203,12 +13203,12 @@
           <t>PIP  127G37</t>
         </is>
       </c>
-      <c r="AT16" t="inlineStr">
+      <c r="AT16" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G46</t>
         </is>
       </c>
-      <c r="AU16" t="inlineStr">
+      <c r="AU16" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G50</t>
         </is>
@@ -13283,12 +13283,12 @@
           <t>CLB GF</t>
         </is>
       </c>
-      <c r="BJ16" t="inlineStr">
+      <c r="BJ16" s="2" t="inlineStr">
         <is>
           <t>CLB GF.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="BK16" t="inlineStr">
+      <c r="BK16" s="2" t="inlineStr">
         <is>
           <t>CLB GF.K MuxBit: 1</t>
         </is>
@@ -13373,12 +13373,12 @@
           <t>CLB GE</t>
         </is>
       </c>
-      <c r="CB16" t="inlineStr">
+      <c r="CB16" s="2" t="inlineStr">
         <is>
           <t>CLB GE.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="CC16" t="inlineStr">
+      <c r="CC16" s="2" t="inlineStr">
         <is>
           <t>CLB GE.K MuxBit: 1</t>
         </is>
@@ -13463,12 +13463,12 @@
           <t>CLB GD</t>
         </is>
       </c>
-      <c r="CT16" t="inlineStr">
+      <c r="CT16" s="2" t="inlineStr">
         <is>
           <t>CLB GD.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="CU16" t="inlineStr">
+      <c r="CU16" s="2" t="inlineStr">
         <is>
           <t>CLB GD.K MuxBit: 1</t>
         </is>
@@ -13483,12 +13483,12 @@
           <t>PIP  67G37</t>
         </is>
       </c>
-      <c r="CX16" t="inlineStr">
+      <c r="CX16" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G46</t>
         </is>
       </c>
-      <c r="CY16" t="inlineStr">
+      <c r="CY16" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G50</t>
         </is>
@@ -13563,12 +13563,12 @@
           <t>CLB GC</t>
         </is>
       </c>
-      <c r="DN16" t="inlineStr">
+      <c r="DN16" s="2" t="inlineStr">
         <is>
           <t>CLB GC.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="DO16" t="inlineStr">
+      <c r="DO16" s="2" t="inlineStr">
         <is>
           <t>CLB GC.K MuxBit: 1</t>
         </is>
@@ -13653,12 +13653,12 @@
           <t>CLB GB</t>
         </is>
       </c>
-      <c r="EF16" t="inlineStr">
+      <c r="EF16" s="2" t="inlineStr">
         <is>
           <t>CLB GB.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="EG16" t="inlineStr">
+      <c r="EG16" s="2" t="inlineStr">
         <is>
           <t>CLB GB.K MuxBit: 1</t>
         </is>
@@ -13743,12 +13743,12 @@
           <t>CLB GA</t>
         </is>
       </c>
-      <c r="EX16" t="inlineStr">
+      <c r="EX16" s="2" t="inlineStr">
         <is>
           <t>CLB GA.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="EY16" t="inlineStr">
+      <c r="EY16" s="2" t="inlineStr">
         <is>
           <t>CLB GA.K MuxBit: 1</t>
         </is>
@@ -16416,7 +16416,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AU20" t="inlineStr">
+      <c r="AU20" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G49</t>
         </is>
@@ -16696,7 +16696,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CY20" t="inlineStr">
+      <c r="CY20" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G49</t>
         </is>
@@ -16993,12 +16993,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Bidi 173G52</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>Bidi 175G52</t>
         </is>
@@ -17028,12 +17028,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>Bidi 176G52</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="J21" s="2" t="inlineStr">
         <is>
           <t>Bidi 151G52</t>
         </is>
@@ -17063,7 +17063,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="P21" t="inlineStr">
+      <c r="P21" s="2" t="inlineStr">
         <is>
           <t>Bidi 150G52</t>
         </is>
@@ -17078,7 +17078,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr">
+      <c r="S21" s="2" t="inlineStr">
         <is>
           <t>Bidi 148G52</t>
         </is>
@@ -17088,7 +17088,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr">
+      <c r="U21" s="2" t="inlineStr">
         <is>
           <t>Bidi 153G52</t>
         </is>
@@ -17118,12 +17118,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AA21" t="inlineStr">
+      <c r="AA21" s="2" t="inlineStr">
         <is>
           <t>Bidi 147G52</t>
         </is>
       </c>
-      <c r="AB21" t="inlineStr">
+      <c r="AB21" s="2" t="inlineStr">
         <is>
           <t>Bidi 131G52</t>
         </is>
@@ -17153,7 +17153,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AH21" t="inlineStr">
+      <c r="AH21" s="2" t="inlineStr">
         <is>
           <t>Bidi 130G52</t>
         </is>
@@ -17168,7 +17168,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AK21" t="inlineStr">
+      <c r="AK21" s="2" t="inlineStr">
         <is>
           <t>Bidi 128G52</t>
         </is>
@@ -17178,7 +17178,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AM21" t="inlineStr">
+      <c r="AM21" s="2" t="inlineStr">
         <is>
           <t>Bidi 133G52</t>
         </is>
@@ -17208,7 +17208,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AS21" t="inlineStr">
+      <c r="AS21" s="2" t="inlineStr">
         <is>
           <t>Bidi 127G52</t>
         </is>
@@ -17223,7 +17223,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AV21" t="inlineStr">
+      <c r="AV21" s="2" t="inlineStr">
         <is>
           <t>Bidi 111G52</t>
         </is>
@@ -17253,7 +17253,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="BB21" t="inlineStr">
+      <c r="BB21" s="2" t="inlineStr">
         <is>
           <t>Bidi 110G52</t>
         </is>
@@ -17268,7 +17268,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="BE21" t="inlineStr">
+      <c r="BE21" s="2" t="inlineStr">
         <is>
           <t>Bidi 108G52</t>
         </is>
@@ -17278,7 +17278,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="BG21" t="inlineStr">
+      <c r="BG21" s="2" t="inlineStr">
         <is>
           <t>Bidi 113G52</t>
         </is>
@@ -17308,12 +17308,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="BM21" t="inlineStr">
+      <c r="BM21" s="2" t="inlineStr">
         <is>
           <t>Bidi 107G52</t>
         </is>
       </c>
-      <c r="BN21" t="inlineStr">
+      <c r="BN21" s="2" t="inlineStr">
         <is>
           <t>Bidi 91G52</t>
         </is>
@@ -17343,7 +17343,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="BT21" t="inlineStr">
+      <c r="BT21" s="2" t="inlineStr">
         <is>
           <t>Bidi 90G52</t>
         </is>
@@ -17358,7 +17358,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="BW21" t="inlineStr">
+      <c r="BW21" s="2" t="inlineStr">
         <is>
           <t>Bidi 88G52</t>
         </is>
@@ -17368,7 +17368,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="BY21" t="inlineStr">
+      <c r="BY21" s="2" t="inlineStr">
         <is>
           <t>Bidi 93G52</t>
         </is>
@@ -17398,12 +17398,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CE21" t="inlineStr">
+      <c r="CE21" s="2" t="inlineStr">
         <is>
           <t>Bidi 87G52</t>
         </is>
       </c>
-      <c r="CF21" t="inlineStr">
+      <c r="CF21" s="2" t="inlineStr">
         <is>
           <t>Bidi 71G52</t>
         </is>
@@ -17433,7 +17433,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CL21" t="inlineStr">
+      <c r="CL21" s="2" t="inlineStr">
         <is>
           <t>Bidi 70G52</t>
         </is>
@@ -17448,7 +17448,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CO21" t="inlineStr">
+      <c r="CO21" s="2" t="inlineStr">
         <is>
           <t>Bidi 68G52</t>
         </is>
@@ -17458,7 +17458,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CQ21" t="inlineStr">
+      <c r="CQ21" s="2" t="inlineStr">
         <is>
           <t>Bidi 73G52</t>
         </is>
@@ -17488,7 +17488,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CW21" t="inlineStr">
+      <c r="CW21" s="2" t="inlineStr">
         <is>
           <t>Bidi 67G52</t>
         </is>
@@ -17503,7 +17503,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CZ21" t="inlineStr">
+      <c r="CZ21" s="2" t="inlineStr">
         <is>
           <t>Bidi 51G52</t>
         </is>
@@ -17533,7 +17533,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="DF21" t="inlineStr">
+      <c r="DF21" s="2" t="inlineStr">
         <is>
           <t>Bidi 50G52</t>
         </is>
@@ -17548,7 +17548,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="DI21" t="inlineStr">
+      <c r="DI21" s="2" t="inlineStr">
         <is>
           <t>Bidi 48G52</t>
         </is>
@@ -17558,7 +17558,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="DK21" t="inlineStr">
+      <c r="DK21" s="2" t="inlineStr">
         <is>
           <t>Bidi 53G52</t>
         </is>
@@ -17588,12 +17588,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="DQ21" t="inlineStr">
+      <c r="DQ21" s="2" t="inlineStr">
         <is>
           <t>Bidi 47G52</t>
         </is>
       </c>
-      <c r="DR21" t="inlineStr">
+      <c r="DR21" s="2" t="inlineStr">
         <is>
           <t>Bidi 31G52</t>
         </is>
@@ -17623,7 +17623,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="DX21" t="inlineStr">
+      <c r="DX21" s="2" t="inlineStr">
         <is>
           <t>Bidi 30G52</t>
         </is>
@@ -17638,7 +17638,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EA21" t="inlineStr">
+      <c r="EA21" s="2" t="inlineStr">
         <is>
           <t>Bidi 28G52</t>
         </is>
@@ -17648,7 +17648,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EC21" t="inlineStr">
+      <c r="EC21" s="2" t="inlineStr">
         <is>
           <t>Bidi 33G52</t>
         </is>
@@ -17678,12 +17678,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EI21" t="inlineStr">
+      <c r="EI21" s="2" t="inlineStr">
         <is>
           <t>Bidi 27G52</t>
         </is>
       </c>
-      <c r="EJ21" t="inlineStr">
+      <c r="EJ21" s="2" t="inlineStr">
         <is>
           <t>Bidi 9G52</t>
         </is>
@@ -17713,7 +17713,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EP21" t="inlineStr">
+      <c r="EP21" s="2" t="inlineStr">
         <is>
           <t>Bidi 8G52</t>
         </is>
@@ -17728,7 +17728,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="ES21" t="inlineStr">
+      <c r="ES21" s="2" t="inlineStr">
         <is>
           <t>Bidi 6G52</t>
         </is>
@@ -17768,7 +17768,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="FA21" t="inlineStr">
+      <c r="FA21" s="2" t="inlineStr">
         <is>
           <t>Bidi 5G52</t>
         </is>
@@ -17790,7 +17790,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>Bidi 172G52</t>
         </is>
@@ -18015,7 +18015,7 @@
           <t>CLB FG Logic Table: 1 Bit: 1</t>
         </is>
       </c>
-      <c r="AT22" t="inlineStr">
+      <c r="AT22" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G66</t>
         </is>
@@ -18295,7 +18295,7 @@
           <t>CLB FD Logic Table: 1 Bit: 1</t>
         </is>
       </c>
-      <c r="CX22" t="inlineStr">
+      <c r="CX22" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G66</t>
         </is>
@@ -20311,12 +20311,12 @@
           <t>CLB FH</t>
         </is>
       </c>
-      <c r="X25" t="inlineStr">
+      <c r="X25" s="2" t="inlineStr">
         <is>
           <t>CLB FH.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="Y25" t="inlineStr">
+      <c r="Y25" s="2" t="inlineStr">
         <is>
           <t>CLB FH.K MuxBit: 1</t>
         </is>
@@ -20401,12 +20401,12 @@
           <t>CLB FG</t>
         </is>
       </c>
-      <c r="AP25" t="inlineStr">
+      <c r="AP25" s="2" t="inlineStr">
         <is>
           <t>CLB FG.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="AQ25" t="inlineStr">
+      <c r="AQ25" s="2" t="inlineStr">
         <is>
           <t>CLB FG.K MuxBit: 1</t>
         </is>
@@ -20421,12 +20421,12 @@
           <t>PIP  127G56</t>
         </is>
       </c>
-      <c r="AT25" t="inlineStr">
+      <c r="AT25" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G65</t>
         </is>
       </c>
-      <c r="AU25" t="inlineStr">
+      <c r="AU25" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G69</t>
         </is>
@@ -20501,12 +20501,12 @@
           <t>CLB FF</t>
         </is>
       </c>
-      <c r="BJ25" t="inlineStr">
+      <c r="BJ25" s="2" t="inlineStr">
         <is>
           <t>CLB FF.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="BK25" t="inlineStr">
+      <c r="BK25" s="2" t="inlineStr">
         <is>
           <t>CLB FF.K MuxBit: 1</t>
         </is>
@@ -20591,12 +20591,12 @@
           <t>CLB FE</t>
         </is>
       </c>
-      <c r="CB25" t="inlineStr">
+      <c r="CB25" s="2" t="inlineStr">
         <is>
           <t>CLB FE.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="CC25" t="inlineStr">
+      <c r="CC25" s="2" t="inlineStr">
         <is>
           <t>CLB FE.K MuxBit: 1</t>
         </is>
@@ -20681,12 +20681,12 @@
           <t>CLB FD</t>
         </is>
       </c>
-      <c r="CT25" t="inlineStr">
+      <c r="CT25" s="2" t="inlineStr">
         <is>
           <t>CLB FD.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="CU25" t="inlineStr">
+      <c r="CU25" s="2" t="inlineStr">
         <is>
           <t>CLB FD.K MuxBit: 1</t>
         </is>
@@ -20701,12 +20701,12 @@
           <t>PIP  67G56</t>
         </is>
       </c>
-      <c r="CX25" t="inlineStr">
+      <c r="CX25" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G65</t>
         </is>
       </c>
-      <c r="CY25" t="inlineStr">
+      <c r="CY25" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G69</t>
         </is>
@@ -20781,12 +20781,12 @@
           <t>CLB FC</t>
         </is>
       </c>
-      <c r="DN25" t="inlineStr">
+      <c r="DN25" s="2" t="inlineStr">
         <is>
           <t>CLB FC.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="DO25" t="inlineStr">
+      <c r="DO25" s="2" t="inlineStr">
         <is>
           <t>CLB FC.K MuxBit: 1</t>
         </is>
@@ -20871,12 +20871,12 @@
           <t>CLB FB</t>
         </is>
       </c>
-      <c r="EF25" t="inlineStr">
+      <c r="EF25" s="2" t="inlineStr">
         <is>
           <t>CLB FB.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="EG25" t="inlineStr">
+      <c r="EG25" s="2" t="inlineStr">
         <is>
           <t>CLB FB.K MuxBit: 1</t>
         </is>
@@ -20961,12 +20961,12 @@
           <t>CLB FA</t>
         </is>
       </c>
-      <c r="EX25" t="inlineStr">
+      <c r="EX25" s="2" t="inlineStr">
         <is>
           <t>CLB FA.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="EY25" t="inlineStr">
+      <c r="EY25" s="2" t="inlineStr">
         <is>
           <t>CLB FA.K MuxBit: 1</t>
         </is>
@@ -23634,7 +23634,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AU29" t="inlineStr">
+      <c r="AU29" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G68</t>
         </is>
@@ -23914,7 +23914,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CY29" t="inlineStr">
+      <c r="CY29" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G68</t>
         </is>
@@ -24431,7 +24431,7 @@
           <t>CLB EG Logic Table: 1 Bit: 1</t>
         </is>
       </c>
-      <c r="AT30" t="inlineStr">
+      <c r="AT30" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G85</t>
         </is>
@@ -24711,7 +24711,7 @@
           <t>CLB ED Logic Table: 1 Bit: 1</t>
         </is>
       </c>
-      <c r="CX30" t="inlineStr">
+      <c r="CX30" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G85</t>
         </is>
@@ -26727,12 +26727,12 @@
           <t>CLB EH</t>
         </is>
       </c>
-      <c r="X33" t="inlineStr">
+      <c r="X33" s="2" t="inlineStr">
         <is>
           <t>CLB EH.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="Y33" t="inlineStr">
+      <c r="Y33" s="2" t="inlineStr">
         <is>
           <t>CLB EH.K MuxBit: 1</t>
         </is>
@@ -26817,12 +26817,12 @@
           <t>CLB EG</t>
         </is>
       </c>
-      <c r="AP33" t="inlineStr">
+      <c r="AP33" s="2" t="inlineStr">
         <is>
           <t>CLB EG.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="AQ33" t="inlineStr">
+      <c r="AQ33" s="2" t="inlineStr">
         <is>
           <t>CLB EG.K MuxBit: 1</t>
         </is>
@@ -26837,12 +26837,12 @@
           <t>PIP  127G75</t>
         </is>
       </c>
-      <c r="AT33" t="inlineStr">
+      <c r="AT33" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G84</t>
         </is>
       </c>
-      <c r="AU33" t="inlineStr">
+      <c r="AU33" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G88</t>
         </is>
@@ -26917,12 +26917,12 @@
           <t>CLB EF</t>
         </is>
       </c>
-      <c r="BJ33" t="inlineStr">
+      <c r="BJ33" s="2" t="inlineStr">
         <is>
           <t>CLB EF.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="BK33" t="inlineStr">
+      <c r="BK33" s="2" t="inlineStr">
         <is>
           <t>CLB EF.K MuxBit: 1</t>
         </is>
@@ -27007,12 +27007,12 @@
           <t>CLB EE</t>
         </is>
       </c>
-      <c r="CB33" t="inlineStr">
+      <c r="CB33" s="2" t="inlineStr">
         <is>
           <t>CLB EE.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="CC33" t="inlineStr">
+      <c r="CC33" s="2" t="inlineStr">
         <is>
           <t>CLB EE.K MuxBit: 1</t>
         </is>
@@ -27097,12 +27097,12 @@
           <t>CLB ED</t>
         </is>
       </c>
-      <c r="CT33" t="inlineStr">
+      <c r="CT33" s="2" t="inlineStr">
         <is>
           <t>CLB ED.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="CU33" t="inlineStr">
+      <c r="CU33" s="2" t="inlineStr">
         <is>
           <t>CLB ED.K MuxBit: 1</t>
         </is>
@@ -27117,12 +27117,12 @@
           <t>PIP  67G75</t>
         </is>
       </c>
-      <c r="CX33" t="inlineStr">
+      <c r="CX33" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G84</t>
         </is>
       </c>
-      <c r="CY33" t="inlineStr">
+      <c r="CY33" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G88</t>
         </is>
@@ -27197,12 +27197,12 @@
           <t>CLB EC</t>
         </is>
       </c>
-      <c r="DN33" t="inlineStr">
+      <c r="DN33" s="2" t="inlineStr">
         <is>
           <t>CLB EC.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="DO33" t="inlineStr">
+      <c r="DO33" s="2" t="inlineStr">
         <is>
           <t>CLB EC.K MuxBit: 1</t>
         </is>
@@ -27287,12 +27287,12 @@
           <t>CLB EB</t>
         </is>
       </c>
-      <c r="EF33" t="inlineStr">
+      <c r="EF33" s="2" t="inlineStr">
         <is>
           <t>CLB EB.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="EG33" t="inlineStr">
+      <c r="EG33" s="2" t="inlineStr">
         <is>
           <t>CLB EB.K MuxBit: 1</t>
         </is>
@@ -27377,12 +27377,12 @@
           <t>CLB EA</t>
         </is>
       </c>
-      <c r="EX33" t="inlineStr">
+      <c r="EX33" s="2" t="inlineStr">
         <is>
           <t>CLB EA.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="EY33" t="inlineStr">
+      <c r="EY33" s="2" t="inlineStr">
         <is>
           <t>CLB EA.K MuxBit: 1</t>
         </is>
@@ -30050,7 +30050,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AU37" t="inlineStr">
+      <c r="AU37" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G87</t>
         </is>
@@ -30330,7 +30330,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CY37" t="inlineStr">
+      <c r="CY37" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G87</t>
         </is>
@@ -30847,7 +30847,7 @@
           <t>CLB DG Logic Table: 1 Bit: 1</t>
         </is>
       </c>
-      <c r="AT38" t="inlineStr">
+      <c r="AT38" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G104</t>
         </is>
@@ -31127,7 +31127,7 @@
           <t>CLB DD Logic Table: 1 Bit: 1</t>
         </is>
       </c>
-      <c r="CX38" t="inlineStr">
+      <c r="CX38" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G104</t>
         </is>
@@ -33143,12 +33143,12 @@
           <t>CLB DH</t>
         </is>
       </c>
-      <c r="X41" t="inlineStr">
+      <c r="X41" s="2" t="inlineStr">
         <is>
           <t>CLB DH.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="Y41" t="inlineStr">
+      <c r="Y41" s="2" t="inlineStr">
         <is>
           <t>CLB DH.K MuxBit: 1</t>
         </is>
@@ -33233,12 +33233,12 @@
           <t>CLB DG</t>
         </is>
       </c>
-      <c r="AP41" t="inlineStr">
+      <c r="AP41" s="2" t="inlineStr">
         <is>
           <t>CLB DG.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="AQ41" t="inlineStr">
+      <c r="AQ41" s="2" t="inlineStr">
         <is>
           <t>CLB DG.K MuxBit: 1</t>
         </is>
@@ -33253,12 +33253,12 @@
           <t>PIP  127G94</t>
         </is>
       </c>
-      <c r="AT41" t="inlineStr">
+      <c r="AT41" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G103</t>
         </is>
       </c>
-      <c r="AU41" t="inlineStr">
+      <c r="AU41" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G107</t>
         </is>
@@ -33333,12 +33333,12 @@
           <t>CLB DF</t>
         </is>
       </c>
-      <c r="BJ41" t="inlineStr">
+      <c r="BJ41" s="2" t="inlineStr">
         <is>
           <t>CLB DF.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="BK41" t="inlineStr">
+      <c r="BK41" s="2" t="inlineStr">
         <is>
           <t>CLB DF.K MuxBit: 1</t>
         </is>
@@ -33423,12 +33423,12 @@
           <t>CLB DE</t>
         </is>
       </c>
-      <c r="CB41" t="inlineStr">
+      <c r="CB41" s="2" t="inlineStr">
         <is>
           <t>CLB DE.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="CC41" t="inlineStr">
+      <c r="CC41" s="2" t="inlineStr">
         <is>
           <t>CLB DE.K MuxBit: 1</t>
         </is>
@@ -33513,12 +33513,12 @@
           <t>CLB DD</t>
         </is>
       </c>
-      <c r="CT41" t="inlineStr">
+      <c r="CT41" s="2" t="inlineStr">
         <is>
           <t>CLB DD.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="CU41" t="inlineStr">
+      <c r="CU41" s="2" t="inlineStr">
         <is>
           <t>CLB DD.K MuxBit: 1</t>
         </is>
@@ -33533,12 +33533,12 @@
           <t>PIP  67G94</t>
         </is>
       </c>
-      <c r="CX41" t="inlineStr">
+      <c r="CX41" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G103</t>
         </is>
       </c>
-      <c r="CY41" t="inlineStr">
+      <c r="CY41" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G107</t>
         </is>
@@ -33613,12 +33613,12 @@
           <t>CLB DC</t>
         </is>
       </c>
-      <c r="DN41" t="inlineStr">
+      <c r="DN41" s="2" t="inlineStr">
         <is>
           <t>CLB DC.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="DO41" t="inlineStr">
+      <c r="DO41" s="2" t="inlineStr">
         <is>
           <t>CLB DC.K MuxBit: 1</t>
         </is>
@@ -33703,12 +33703,12 @@
           <t>CLB DB</t>
         </is>
       </c>
-      <c r="EF41" t="inlineStr">
+      <c r="EF41" s="2" t="inlineStr">
         <is>
           <t>CLB DB.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="EG41" t="inlineStr">
+      <c r="EG41" s="2" t="inlineStr">
         <is>
           <t>CLB DB.K MuxBit: 1</t>
         </is>
@@ -33793,12 +33793,12 @@
           <t>CLB DA</t>
         </is>
       </c>
-      <c r="EX41" t="inlineStr">
+      <c r="EX41" s="2" t="inlineStr">
         <is>
           <t>CLB DA.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="EY41" t="inlineStr">
+      <c r="EY41" s="2" t="inlineStr">
         <is>
           <t>CLB DA.K MuxBit: 1</t>
         </is>
@@ -36466,7 +36466,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AU45" t="inlineStr">
+      <c r="AU45" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G106</t>
         </is>
@@ -36746,7 +36746,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CY45" t="inlineStr">
+      <c r="CY45" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G106</t>
         </is>
@@ -37043,12 +37043,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>Bidi 173G109</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Bidi 175G109</t>
         </is>
@@ -37078,12 +37078,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="I46" s="2" t="inlineStr">
         <is>
           <t>Bidi 176G109</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="J46" s="2" t="inlineStr">
         <is>
           <t>Bidi 151G109</t>
         </is>
@@ -37113,7 +37113,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="P46" t="inlineStr">
+      <c r="P46" s="2" t="inlineStr">
         <is>
           <t>Bidi 150G109</t>
         </is>
@@ -37128,7 +37128,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="S46" t="inlineStr">
+      <c r="S46" s="2" t="inlineStr">
         <is>
           <t>Bidi 148G109</t>
         </is>
@@ -37138,7 +37138,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="U46" t="inlineStr">
+      <c r="U46" s="2" t="inlineStr">
         <is>
           <t>Bidi 153G109</t>
         </is>
@@ -37168,12 +37168,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AA46" t="inlineStr">
+      <c r="AA46" s="2" t="inlineStr">
         <is>
           <t>Bidi 147G109</t>
         </is>
       </c>
-      <c r="AB46" t="inlineStr">
+      <c r="AB46" s="2" t="inlineStr">
         <is>
           <t>Bidi 131G109</t>
         </is>
@@ -37203,7 +37203,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AH46" t="inlineStr">
+      <c r="AH46" s="2" t="inlineStr">
         <is>
           <t>Bidi 130G109</t>
         </is>
@@ -37218,7 +37218,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AK46" t="inlineStr">
+      <c r="AK46" s="2" t="inlineStr">
         <is>
           <t>Bidi 128G109</t>
         </is>
@@ -37228,7 +37228,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AM46" t="inlineStr">
+      <c r="AM46" s="2" t="inlineStr">
         <is>
           <t>Bidi 133G109</t>
         </is>
@@ -37258,7 +37258,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AS46" t="inlineStr">
+      <c r="AS46" s="2" t="inlineStr">
         <is>
           <t>Bidi 127G109</t>
         </is>
@@ -37273,7 +37273,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AV46" t="inlineStr">
+      <c r="AV46" s="2" t="inlineStr">
         <is>
           <t>Bidi 111G109</t>
         </is>
@@ -37303,7 +37303,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="BB46" t="inlineStr">
+      <c r="BB46" s="2" t="inlineStr">
         <is>
           <t>Bidi 110G109</t>
         </is>
@@ -37318,7 +37318,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="BE46" t="inlineStr">
+      <c r="BE46" s="2" t="inlineStr">
         <is>
           <t>Bidi 108G109</t>
         </is>
@@ -37328,7 +37328,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="BG46" t="inlineStr">
+      <c r="BG46" s="2" t="inlineStr">
         <is>
           <t>Bidi 113G109</t>
         </is>
@@ -37358,12 +37358,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="BM46" t="inlineStr">
+      <c r="BM46" s="2" t="inlineStr">
         <is>
           <t>Bidi 107G109</t>
         </is>
       </c>
-      <c r="BN46" t="inlineStr">
+      <c r="BN46" s="2" t="inlineStr">
         <is>
           <t>Bidi 91G109</t>
         </is>
@@ -37393,7 +37393,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="BT46" t="inlineStr">
+      <c r="BT46" s="2" t="inlineStr">
         <is>
           <t>Bidi 90G109</t>
         </is>
@@ -37408,7 +37408,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="BW46" t="inlineStr">
+      <c r="BW46" s="2" t="inlineStr">
         <is>
           <t>Bidi 88G109</t>
         </is>
@@ -37418,7 +37418,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="BY46" t="inlineStr">
+      <c r="BY46" s="2" t="inlineStr">
         <is>
           <t>Bidi 93G109</t>
         </is>
@@ -37448,12 +37448,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CE46" t="inlineStr">
+      <c r="CE46" s="2" t="inlineStr">
         <is>
           <t>Bidi 87G109</t>
         </is>
       </c>
-      <c r="CF46" t="inlineStr">
+      <c r="CF46" s="2" t="inlineStr">
         <is>
           <t>Bidi 71G109</t>
         </is>
@@ -37483,7 +37483,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CL46" t="inlineStr">
+      <c r="CL46" s="2" t="inlineStr">
         <is>
           <t>Bidi 70G109</t>
         </is>
@@ -37498,7 +37498,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CO46" t="inlineStr">
+      <c r="CO46" s="2" t="inlineStr">
         <is>
           <t>Bidi 68G109</t>
         </is>
@@ -37508,7 +37508,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CQ46" t="inlineStr">
+      <c r="CQ46" s="2" t="inlineStr">
         <is>
           <t>Bidi 73G109</t>
         </is>
@@ -37538,7 +37538,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CW46" t="inlineStr">
+      <c r="CW46" s="2" t="inlineStr">
         <is>
           <t>Bidi 67G109</t>
         </is>
@@ -37553,7 +37553,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CZ46" t="inlineStr">
+      <c r="CZ46" s="2" t="inlineStr">
         <is>
           <t>Bidi 51G109</t>
         </is>
@@ -37583,7 +37583,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="DF46" t="inlineStr">
+      <c r="DF46" s="2" t="inlineStr">
         <is>
           <t>Bidi 50G109</t>
         </is>
@@ -37598,7 +37598,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="DI46" t="inlineStr">
+      <c r="DI46" s="2" t="inlineStr">
         <is>
           <t>Bidi 48G109</t>
         </is>
@@ -37608,7 +37608,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="DK46" t="inlineStr">
+      <c r="DK46" s="2" t="inlineStr">
         <is>
           <t>Bidi 53G109</t>
         </is>
@@ -37638,12 +37638,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="DQ46" t="inlineStr">
+      <c r="DQ46" s="2" t="inlineStr">
         <is>
           <t>Bidi 47G109</t>
         </is>
       </c>
-      <c r="DR46" t="inlineStr">
+      <c r="DR46" s="2" t="inlineStr">
         <is>
           <t>Bidi 31G109</t>
         </is>
@@ -37673,7 +37673,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="DX46" t="inlineStr">
+      <c r="DX46" s="2" t="inlineStr">
         <is>
           <t>Bidi 30G109</t>
         </is>
@@ -37688,7 +37688,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EA46" t="inlineStr">
+      <c r="EA46" s="2" t="inlineStr">
         <is>
           <t>Bidi 28G109</t>
         </is>
@@ -37698,7 +37698,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EC46" t="inlineStr">
+      <c r="EC46" s="2" t="inlineStr">
         <is>
           <t>Bidi 33G109</t>
         </is>
@@ -37728,12 +37728,12 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EI46" t="inlineStr">
+      <c r="EI46" s="2" t="inlineStr">
         <is>
           <t>Bidi 27G109</t>
         </is>
       </c>
-      <c r="EJ46" t="inlineStr">
+      <c r="EJ46" s="2" t="inlineStr">
         <is>
           <t>Bidi 9G109</t>
         </is>
@@ -37763,7 +37763,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="EP46" t="inlineStr">
+      <c r="EP46" s="2" t="inlineStr">
         <is>
           <t>Bidi 8G109</t>
         </is>
@@ -37778,7 +37778,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="ES46" t="inlineStr">
+      <c r="ES46" s="2" t="inlineStr">
         <is>
           <t>Bidi 6G109</t>
         </is>
@@ -37818,7 +37818,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="FA46" t="inlineStr">
+      <c r="FA46" s="2" t="inlineStr">
         <is>
           <t>Bidi 5G109</t>
         </is>
@@ -37840,7 +37840,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>Bidi 172G109</t>
         </is>
@@ -38065,7 +38065,7 @@
           <t>CLB CG Logic Table: 1 Bit: 1</t>
         </is>
       </c>
-      <c r="AT47" t="inlineStr">
+      <c r="AT47" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G123</t>
         </is>
@@ -38345,7 +38345,7 @@
           <t>CLB CD Logic Table: 1 Bit: 1</t>
         </is>
       </c>
-      <c r="CX47" t="inlineStr">
+      <c r="CX47" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G123</t>
         </is>
@@ -40361,12 +40361,12 @@
           <t>CLB CH</t>
         </is>
       </c>
-      <c r="X50" t="inlineStr">
+      <c r="X50" s="2" t="inlineStr">
         <is>
           <t>CLB CH.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="Y50" t="inlineStr">
+      <c r="Y50" s="2" t="inlineStr">
         <is>
           <t>CLB CH.K MuxBit: 1</t>
         </is>
@@ -40451,12 +40451,12 @@
           <t>CLB CG</t>
         </is>
       </c>
-      <c r="AP50" t="inlineStr">
+      <c r="AP50" s="2" t="inlineStr">
         <is>
           <t>CLB CG.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="AQ50" t="inlineStr">
+      <c r="AQ50" s="2" t="inlineStr">
         <is>
           <t>CLB CG.K MuxBit: 1</t>
         </is>
@@ -40471,12 +40471,12 @@
           <t>PIP  127G113</t>
         </is>
       </c>
-      <c r="AT50" t="inlineStr">
+      <c r="AT50" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G122</t>
         </is>
       </c>
-      <c r="AU50" t="inlineStr">
+      <c r="AU50" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G126</t>
         </is>
@@ -40551,12 +40551,12 @@
           <t>CLB CF</t>
         </is>
       </c>
-      <c r="BJ50" t="inlineStr">
+      <c r="BJ50" s="2" t="inlineStr">
         <is>
           <t>CLB CF.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="BK50" t="inlineStr">
+      <c r="BK50" s="2" t="inlineStr">
         <is>
           <t>CLB CF.K MuxBit: 1</t>
         </is>
@@ -40641,12 +40641,12 @@
           <t>CLB CE</t>
         </is>
       </c>
-      <c r="CB50" t="inlineStr">
+      <c r="CB50" s="2" t="inlineStr">
         <is>
           <t>CLB CE.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="CC50" t="inlineStr">
+      <c r="CC50" s="2" t="inlineStr">
         <is>
           <t>CLB CE.K MuxBit: 1</t>
         </is>
@@ -40731,12 +40731,12 @@
           <t>CLB CD</t>
         </is>
       </c>
-      <c r="CT50" t="inlineStr">
+      <c r="CT50" s="2" t="inlineStr">
         <is>
           <t>CLB CD.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="CU50" t="inlineStr">
+      <c r="CU50" s="2" t="inlineStr">
         <is>
           <t>CLB CD.K MuxBit: 1</t>
         </is>
@@ -40751,12 +40751,12 @@
           <t>PIP  67G113</t>
         </is>
       </c>
-      <c r="CX50" t="inlineStr">
+      <c r="CX50" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G122</t>
         </is>
       </c>
-      <c r="CY50" t="inlineStr">
+      <c r="CY50" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G126</t>
         </is>
@@ -40831,12 +40831,12 @@
           <t>CLB CC</t>
         </is>
       </c>
-      <c r="DN50" t="inlineStr">
+      <c r="DN50" s="2" t="inlineStr">
         <is>
           <t>CLB CC.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="DO50" t="inlineStr">
+      <c r="DO50" s="2" t="inlineStr">
         <is>
           <t>CLB CC.K MuxBit: 1</t>
         </is>
@@ -40921,12 +40921,12 @@
           <t>CLB CB</t>
         </is>
       </c>
-      <c r="EF50" t="inlineStr">
+      <c r="EF50" s="2" t="inlineStr">
         <is>
           <t>CLB CB.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="EG50" t="inlineStr">
+      <c r="EG50" s="2" t="inlineStr">
         <is>
           <t>CLB CB.K MuxBit: 1</t>
         </is>
@@ -41011,12 +41011,12 @@
           <t>CLB CA</t>
         </is>
       </c>
-      <c r="EX50" t="inlineStr">
+      <c r="EX50" s="2" t="inlineStr">
         <is>
           <t>CLB CA.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="EY50" t="inlineStr">
+      <c r="EY50" s="2" t="inlineStr">
         <is>
           <t>CLB CA.K MuxBit: 1</t>
         </is>
@@ -43684,7 +43684,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AU54" t="inlineStr">
+      <c r="AU54" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G125</t>
         </is>
@@ -43964,7 +43964,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CY54" t="inlineStr">
+      <c r="CY54" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G125</t>
         </is>
@@ -44481,7 +44481,7 @@
           <t>CLB BG Logic Table: 1 Bit: 1</t>
         </is>
       </c>
-      <c r="AT55" t="inlineStr">
+      <c r="AT55" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G142</t>
         </is>
@@ -44761,7 +44761,7 @@
           <t>CLB BD Logic Table: 1 Bit: 1</t>
         </is>
       </c>
-      <c r="CX55" t="inlineStr">
+      <c r="CX55" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G142</t>
         </is>
@@ -46777,12 +46777,12 @@
           <t>CLB BH</t>
         </is>
       </c>
-      <c r="X58" t="inlineStr">
+      <c r="X58" s="2" t="inlineStr">
         <is>
           <t>CLB BH.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="Y58" t="inlineStr">
+      <c r="Y58" s="2" t="inlineStr">
         <is>
           <t>CLB BH.K MuxBit: 1</t>
         </is>
@@ -46867,12 +46867,12 @@
           <t>CLB BG</t>
         </is>
       </c>
-      <c r="AP58" t="inlineStr">
+      <c r="AP58" s="2" t="inlineStr">
         <is>
           <t>CLB BG.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="AQ58" t="inlineStr">
+      <c r="AQ58" s="2" t="inlineStr">
         <is>
           <t>CLB BG.K MuxBit: 1</t>
         </is>
@@ -46887,12 +46887,12 @@
           <t>PIP  127G132</t>
         </is>
       </c>
-      <c r="AT58" t="inlineStr">
+      <c r="AT58" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G141</t>
         </is>
       </c>
-      <c r="AU58" t="inlineStr">
+      <c r="AU58" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G145</t>
         </is>
@@ -46967,12 +46967,12 @@
           <t>CLB BF</t>
         </is>
       </c>
-      <c r="BJ58" t="inlineStr">
+      <c r="BJ58" s="2" t="inlineStr">
         <is>
           <t>CLB BF.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="BK58" t="inlineStr">
+      <c r="BK58" s="2" t="inlineStr">
         <is>
           <t>CLB BF.K MuxBit: 1</t>
         </is>
@@ -47057,12 +47057,12 @@
           <t>CLB BE</t>
         </is>
       </c>
-      <c r="CB58" t="inlineStr">
+      <c r="CB58" s="2" t="inlineStr">
         <is>
           <t>CLB BE.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="CC58" t="inlineStr">
+      <c r="CC58" s="2" t="inlineStr">
         <is>
           <t>CLB BE.K MuxBit: 1</t>
         </is>
@@ -47147,12 +47147,12 @@
           <t>CLB BD</t>
         </is>
       </c>
-      <c r="CT58" t="inlineStr">
+      <c r="CT58" s="2" t="inlineStr">
         <is>
           <t>CLB BD.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="CU58" t="inlineStr">
+      <c r="CU58" s="2" t="inlineStr">
         <is>
           <t>CLB BD.K MuxBit: 1</t>
         </is>
@@ -47167,12 +47167,12 @@
           <t>PIP  67G132</t>
         </is>
       </c>
-      <c r="CX58" t="inlineStr">
+      <c r="CX58" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G141</t>
         </is>
       </c>
-      <c r="CY58" t="inlineStr">
+      <c r="CY58" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G145</t>
         </is>
@@ -47247,12 +47247,12 @@
           <t>CLB BC</t>
         </is>
       </c>
-      <c r="DN58" t="inlineStr">
+      <c r="DN58" s="2" t="inlineStr">
         <is>
           <t>CLB BC.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="DO58" t="inlineStr">
+      <c r="DO58" s="2" t="inlineStr">
         <is>
           <t>CLB BC.K MuxBit: 1</t>
         </is>
@@ -47337,12 +47337,12 @@
           <t>CLB BB</t>
         </is>
       </c>
-      <c r="EF58" t="inlineStr">
+      <c r="EF58" s="2" t="inlineStr">
         <is>
           <t>CLB BB.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="EG58" t="inlineStr">
+      <c r="EG58" s="2" t="inlineStr">
         <is>
           <t>CLB BB.K MuxBit: 1</t>
         </is>
@@ -47427,12 +47427,12 @@
           <t>CLB BA</t>
         </is>
       </c>
-      <c r="EX58" t="inlineStr">
+      <c r="EX58" s="2" t="inlineStr">
         <is>
           <t>CLB BA.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="EY58" t="inlineStr">
+      <c r="EY58" s="2" t="inlineStr">
         <is>
           <t>CLB BA.K MuxBit: 1</t>
         </is>
@@ -50100,7 +50100,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AU62" t="inlineStr">
+      <c r="AU62" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G144</t>
         </is>
@@ -50380,7 +50380,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CY62" t="inlineStr">
+      <c r="CY62" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G144</t>
         </is>
@@ -53193,12 +53193,12 @@
           <t>CLB AH</t>
         </is>
       </c>
-      <c r="X66" t="inlineStr">
+      <c r="X66" s="2" t="inlineStr">
         <is>
           <t>CLB AH.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="Y66" t="inlineStr">
+      <c r="Y66" s="2" t="inlineStr">
         <is>
           <t>CLB AH.K MuxBit: 1</t>
         </is>
@@ -53283,12 +53283,12 @@
           <t>CLB AG</t>
         </is>
       </c>
-      <c r="AP66" t="inlineStr">
+      <c r="AP66" s="2" t="inlineStr">
         <is>
           <t>CLB AG.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="AQ66" t="inlineStr">
+      <c r="AQ66" s="2" t="inlineStr">
         <is>
           <t>CLB AG.K MuxBit: 1</t>
         </is>
@@ -53383,12 +53383,12 @@
           <t>CLB AF</t>
         </is>
       </c>
-      <c r="BJ66" t="inlineStr">
+      <c r="BJ66" s="2" t="inlineStr">
         <is>
           <t>CLB AF.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="BK66" t="inlineStr">
+      <c r="BK66" s="2" t="inlineStr">
         <is>
           <t>CLB AF.K MuxBit: 1</t>
         </is>
@@ -53473,12 +53473,12 @@
           <t>CLB AE</t>
         </is>
       </c>
-      <c r="CB66" t="inlineStr">
+      <c r="CB66" s="2" t="inlineStr">
         <is>
           <t>CLB AE.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="CC66" t="inlineStr">
+      <c r="CC66" s="2" t="inlineStr">
         <is>
           <t>CLB AE.K MuxBit: 1</t>
         </is>
@@ -53563,12 +53563,12 @@
           <t>CLB AD</t>
         </is>
       </c>
-      <c r="CT66" t="inlineStr">
+      <c r="CT66" s="2" t="inlineStr">
         <is>
           <t>CLB AD.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="CU66" t="inlineStr">
+      <c r="CU66" s="2" t="inlineStr">
         <is>
           <t>CLB AD.K MuxBit: 1</t>
         </is>
@@ -53663,12 +53663,12 @@
           <t>CLB AC</t>
         </is>
       </c>
-      <c r="DN66" t="inlineStr">
+      <c r="DN66" s="2" t="inlineStr">
         <is>
           <t>CLB AC.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="DO66" t="inlineStr">
+      <c r="DO66" s="2" t="inlineStr">
         <is>
           <t>CLB AC.K MuxBit: 1</t>
         </is>
@@ -53753,12 +53753,12 @@
           <t>CLB AB</t>
         </is>
       </c>
-      <c r="EF66" t="inlineStr">
+      <c r="EF66" s="2" t="inlineStr">
         <is>
           <t>CLB AB.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="EG66" t="inlineStr">
+      <c r="EG66" s="2" t="inlineStr">
         <is>
           <t>CLB AB.K MuxBit: 1</t>
         </is>
@@ -53843,12 +53843,12 @@
           <t>CLB AA</t>
         </is>
       </c>
-      <c r="EX66" t="inlineStr">
+      <c r="EX66" s="2" t="inlineStr">
         <is>
           <t>CLB AA.K MuxBit: 0</t>
         </is>
       </c>
-      <c r="EY66" t="inlineStr">
+      <c r="EY66" s="2" t="inlineStr">
         <is>
           <t>CLB AA.K MuxBit: 1</t>
         </is>
@@ -54105,7 +54105,7 @@
           <t>CLB AG.C MuxBit: 3</t>
         </is>
       </c>
-      <c r="AT67" t="inlineStr">
+      <c r="AT67" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G163</t>
         </is>
@@ -54385,7 +54385,7 @@
           <t>CLB AD.C MuxBit: 3</t>
         </is>
       </c>
-      <c r="CX67" t="inlineStr">
+      <c r="CX67" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G163</t>
         </is>
@@ -56516,7 +56516,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="AU70" t="inlineStr">
+      <c r="AU70" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G164</t>
         </is>
@@ -56796,7 +56796,7 @@
           <t>----- NOT USED -----</t>
         </is>
       </c>
-      <c r="CY70" t="inlineStr">
+      <c r="CY70" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G164</t>
         </is>
@@ -57308,12 +57308,12 @@
           <t>IOB P64.O MuxBit: 3</t>
         </is>
       </c>
-      <c r="AT71" t="inlineStr">
+      <c r="AT71" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G167</t>
         </is>
       </c>
-      <c r="AU71" t="inlineStr">
+      <c r="AU71" s="2" t="inlineStr">
         <is>
           <t>Bidi 125G166</t>
         </is>
@@ -57588,12 +57588,12 @@
           <t>IOB P3.O MuxBit: 3</t>
         </is>
       </c>
-      <c r="CX71" t="inlineStr">
+      <c r="CX71" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G167</t>
         </is>
       </c>
-      <c r="CY71" t="inlineStr">
+      <c r="CY71" s="2" t="inlineStr">
         <is>
           <t>Bidi 65G166</t>
         </is>

</xml_diff>